<commit_message>
feat: Enhance WWTP WCO Data API with lazy loading support for sections
- Added support for lazy loading of specific sections in the wwtp_wco_data method.
- Introduced a new query parameter `section` to fetch data for specific sections like 'biaya', 'analisa', 'status_operasi', etc.
- Refactored data retrieval methods to streamline responses based on the requested section.
- Updated the dashboard view to accommodate changes in the TSS compliance card, allowing for fallback to HSE training data.
- Improved overall response structure for better clarity and maintainability.
</commit_message>
<xml_diff>
--- a/public/assets/templates/operasional/mdp.xlsx
+++ b/public/assets/templates/operasional/mdp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\operasional\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98D5229B-A533-40B3-80D8-59FD83500C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8E20C6C-9999-4DEB-AC64-943175B67D08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{48748F47-9D71-4608-BC1F-023F595FFB4F}"/>
   </bookViews>
@@ -114,10 +114,10 @@
     <t>Suhu Ruang</t>
   </si>
   <si>
-    <t>Trafo</t>
-  </si>
-  <si>
-    <t>Genset</t>
+    <t>Trafo (°C)</t>
+  </si>
+  <si>
+    <t>Genset (°C)</t>
   </si>
 </sst>
 </file>
@@ -540,64 +540,64 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -967,22 +967,22 @@
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:21" ht="15" thickTop="1">
-      <c r="A1" s="31"/>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="35" t="s">
+      <c r="A1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
       <c r="O1" s="1" t="s">
         <v>1</v>
       </c>
@@ -994,22 +994,22 @@
       <c r="U1" s="4"/>
     </row>
     <row r="2" spans="1:21">
-      <c r="A2" s="33"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="37" t="s">
+      <c r="A2" s="26"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="38"/>
-      <c r="L2" s="38"/>
-      <c r="M2" s="38"/>
-      <c r="N2" s="38"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
       <c r="O2" s="7" t="s">
         <v>3</v>
       </c>
@@ -1021,59 +1021,59 @@
       <c r="U2" s="10"/>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="23" t="s">
+      <c r="E3" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="24"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="21" t="s">
+      <c r="F3" s="22"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="23" t="s">
+      <c r="I3" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="24"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="21" t="s">
+      <c r="J3" s="22"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="M3" s="23" t="s">
+      <c r="M3" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="N3" s="24"/>
-      <c r="O3" s="24"/>
-      <c r="P3" s="25" t="s">
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="Q3" s="25"/>
-      <c r="R3" s="25" t="s">
+      <c r="Q3" s="38"/>
+      <c r="R3" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="S3" s="25"/>
-      <c r="T3" s="26" t="s">
+      <c r="S3" s="38"/>
+      <c r="T3" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="U3" s="28" t="s">
+      <c r="U3" s="39" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="26">
-      <c r="A4" s="40"/>
-      <c r="B4" s="27"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
+      <c r="A4" s="33"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
       <c r="E4" s="6" t="s">
         <v>16</v>
       </c>
@@ -1083,7 +1083,7 @@
       <c r="G4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="22"/>
+      <c r="H4" s="37"/>
       <c r="I4" s="6" t="s">
         <v>19</v>
       </c>
@@ -1093,7 +1093,7 @@
       <c r="K4" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="L4" s="22"/>
+      <c r="L4" s="37"/>
       <c r="M4" s="6" t="s">
         <v>22</v>
       </c>
@@ -1115,8 +1115,8 @@
       <c r="S4" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="T4" s="27"/>
-      <c r="U4" s="29"/>
+      <c r="T4" s="35"/>
+      <c r="U4" s="40"/>
     </row>
     <row r="5" spans="1:21">
       <c r="A5" s="5">
@@ -1920,6 +1920,10 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="U3:U4"/>
+    <mergeCell ref="R3:S3"/>
     <mergeCell ref="I3:K3"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="D1:N1"/>
@@ -1932,10 +1936,6 @@
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="M3:O3"/>
-    <mergeCell ref="P3:Q3"/>
-    <mergeCell ref="T3:T4"/>
-    <mergeCell ref="U3:U4"/>
-    <mergeCell ref="R3:S3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>